<commit_message>
fix(presupuesto): actualizar P-2026-0047 cliente, confirming 90 dias y precios unitarios 01, 04 y 06
</commit_message>
<xml_diff>
--- a/presupuestos/P-2026-0047-partidas-hotel-sur-2026-2027/presupuesto.xlsx
+++ b/presupuestos/P-2026-0047-partidas-hotel-sur-2026-2027/presupuesto.xlsx
@@ -516,7 +516,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>PRESUPUESTO TÉCNICO Y ECONÓMICO: P-2026-0047</t>
+          <t>PRESUPUESTO TÉCNICO Y ECONÓMICO: P-2026-0047 (REV. 1)</t>
         </is>
       </c>
     </row>
@@ -528,19 +528,19 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Hotel Sur</t>
+          <t>PROMOCION Y DESARROLLO TURISTICO DE MENORCA SOCIEDAD LIMITADA</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Ubicación:</t>
+          <t>Establecimiento / Obra:</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Instalaciones Hotel Sur, Menorca</t>
+          <t>Hotel Sur, Menorca</t>
         </is>
       </c>
     </row>
@@ -571,12 +571,12 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Período Previsto:</t>
+          <t>Forma de Pago:</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Temporada baja hotelera 2026 / 2027</t>
+          <t>Confirming 90 días</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>6 partidas completas de renovación. Incluye desmontaje y retirada de elementos antiguos en partidas 2, 3, 4 y 6. Materiales de alta resistencia al ambiente marino (Inox AISI 316L, aluminio Qualicoat y vidrio de seguridad).</t>
+          <t>6 partidas de renovación integral. Incluye desmontaje y retirada de viejos elementos en partidas 2, 3, 4 y 6. Calidad marina Inox AISI 316L, aluminio Qualicoat y vidrio laminar de seguridad. Pago mediante Confirming 90 días.</t>
         </is>
       </c>
     </row>
@@ -644,10 +644,10 @@
         <v>13.9392</v>
       </c>
       <c r="E13" s="12" t="n">
-        <v>400</v>
+        <v>403.21</v>
       </c>
       <c r="F13" s="12">
-        <f>D13*E13</f>
+        <f>ROUND(D13*E13, 2)</f>
         <v/>
       </c>
     </row>
@@ -674,7 +674,7 @@
         <v>455</v>
       </c>
       <c r="F14" s="12">
-        <f>D14*E14</f>
+        <f>ROUND(D14*E14, 2)</f>
         <v/>
       </c>
     </row>
@@ -701,7 +701,7 @@
         <v>2300</v>
       </c>
       <c r="F15" s="12">
-        <f>D15*E15</f>
+        <f>ROUND(D15*E15, 2)</f>
         <v/>
       </c>
     </row>
@@ -725,10 +725,10 @@
         <v>13.5</v>
       </c>
       <c r="E16" s="12" t="n">
-        <v>330</v>
+        <v>333.14</v>
       </c>
       <c r="F16" s="12">
-        <f>D16*E16</f>
+        <f>ROUND(D16*E16, 2)</f>
         <v/>
       </c>
     </row>
@@ -755,7 +755,7 @@
         <v>1250</v>
       </c>
       <c r="F17" s="12">
-        <f>D17*E17</f>
+        <f>ROUND(D17*E17, 2)</f>
         <v/>
       </c>
     </row>
@@ -779,10 +779,10 @@
         <v>3</v>
       </c>
       <c r="E18" s="12" t="n">
-        <v>500</v>
+        <v>497.12</v>
       </c>
       <c r="F18" s="12">
-        <f>D18*E18</f>
+        <f>ROUND(D18*E18, 2)</f>
         <v/>
       </c>
     </row>
@@ -804,7 +804,7 @@
         </is>
       </c>
       <c r="F21" s="14">
-        <f>F20*0.21</f>
+        <f>ROUND(F20*0.21, 2)</f>
         <v/>
       </c>
     </row>

</xml_diff>